<commit_message>
Add rudder metrics and reverse-rudder detection
</commit_message>
<xml_diff>
--- a/result_sample/result_sample.xlsx
+++ b/result_sample/result_sample.xlsx
@@ -1,99 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cqueducn0-my.sharepoint.com/personal/20162719_cqu_edu_cn/Documents/飞行资料/CA/飞行部/QAR/result_sample/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_AD4DA82427541F7ACA7EB843700D0E126AE8DE12" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D25324E-475B-4FA8-9C25-5E0E1783995F}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="2370" windowWidth="24315" windowHeight="18300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="7200" yWindow="2370" windowWidth="24315" windowHeight="18300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="162913" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>低空 300ft AGL 以下杆量超过 15 个单位次数</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>低空 300ft AGL 以下杆量超过 15 个单位占比</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>低空 50ft AGL 以下舵量超过 15 个单位次数</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>低空 50ft AGL 以下舵量超过 15 个单位占比</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>接地交叉角大于 6° 占比</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>接地交叉角大于 6° 次数</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>高高原次数</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>高高原占比</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>姓名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve"> PF 抬头速率大于 3.5°/s 占比</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve"> PF 抬头速率大于 3.5°/s 次数</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="等线"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="9"/>
-      <name val="等线"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -112,24 +53,83 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -395,54 +395,86 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="2" width="10.625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.625" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="9" style="1"/>
+    <col width="9" customWidth="1" style="1" min="1" max="1"/>
+    <col width="10.625" customWidth="1" style="1" min="2" max="2"/>
+    <col width="9.875" customWidth="1" style="1" min="3" max="3"/>
+    <col width="10.625" customWidth="1" style="1" min="4" max="4"/>
+    <col width="9" customWidth="1" style="1" min="5" max="16384"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>7</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>低空 300ft AGL 以下杆量超过 15 个单位次数</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>低空 300ft AGL 以下杆量超过 15 个单位占比</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>低空 50ft AGL 以下舵量超过 15 个单位次数</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>低空 50ft AGL 以下舵量超过 15 个单位占比</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>接地交叉角大于 6° 次数</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>接地交叉角大于 6° 占比</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PF 抬头速率大于 3.5°/s 次数</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> PF 抬头速率大于 3.5°/s 占比</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>高高原次数</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>高高原占比</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>疑似接地前反向蹬舵次数</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add aircraft database classification and report links
</commit_message>
<xml_diff>
--- a/result_sample/result_sample.xlsx
+++ b/result_sample/result_sample.xlsx
@@ -1,40 +1,105 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cqueducn0-my.sharepoint.com/personal/20162719_cqu_edu_cn/Documents/飞行资料/CA/飞行部/QAR/result_sample/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_66E65D56D24B0A4F6A7984F55289D6394056AD5C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58AAA9DE-83DB-4296-AE39-8EEC66D92373}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="7200" yWindow="2370" windowWidth="24315" windowHeight="18300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="3510" yWindow="3300" windowWidth="24315" windowHeight="18300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="162913" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t>姓名</t>
+  </si>
+  <si>
+    <t>低空 300ft AGL 以下杆量超过 15 个单位采样点数</t>
+  </si>
+  <si>
+    <t>低空 300ft AGL 以下杆量超过 15 个单位采样点占比</t>
+  </si>
+  <si>
+    <t>低空 50ft AGL 以下舵量超过 15 个单位次数</t>
+  </si>
+  <si>
+    <t>低空 50ft AGL 以下舵量超过 15 个单位占比</t>
+  </si>
+  <si>
+    <t>接地交叉角大于 6° 次数</t>
+  </si>
+  <si>
+    <t>接地交叉角大于 6° 占比</t>
+  </si>
+  <si>
+    <t>PF 抬头速率大于 3.5°/s 次数</t>
+  </si>
+  <si>
+    <t>PF 抬头速率大于 3.5°/s 占比</t>
+  </si>
+  <si>
+    <t>抬头速率大中高高原次数</t>
+  </si>
+  <si>
+    <t>抬头速率大中高高原占比</t>
+  </si>
+  <si>
+    <t>疑似接地前反向蹬舵次数</t>
+  </si>
+  <si>
+    <t>何玺</t>
+  </si>
+  <si>
+    <t>机型</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A319</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A320,A321</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A321NEO</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="等线"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9"/>
       <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
-      <family val="3"/>
-      <sz val="9"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -52,84 +117,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -395,86 +408,368 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:M17"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col width="9" customWidth="1" style="1" min="1" max="1"/>
-    <col width="10.625" customWidth="1" style="1" min="2" max="2"/>
-    <col width="9.875" customWidth="1" style="1" min="3" max="3"/>
-    <col width="10.625" customWidth="1" style="1" min="4" max="4"/>
-    <col width="9" customWidth="1" style="1" min="5" max="16384"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
+    <col min="1" max="1" width="9" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="10.625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9" style="1" customWidth="1"/>
+    <col min="7" max="11" width="9" style="1"/>
+    <col min="12" max="13" width="13" customWidth="1"/>
+    <col min="14" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>姓名</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>低空 300ft AGL 以下杆量超过 15 个单位次数</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>低空 300ft AGL 以下杆量超过 15 个单位占比</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>低空 50ft AGL 以下舵量超过 15 个单位次数</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>低空 50ft AGL 以下舵量超过 15 个单位占比</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>接地交叉角大于 6° 次数</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>接地交叉角大于 6° 占比</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> PF 抬头速率大于 3.5°/s 次数</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> PF 抬头速率大于 3.5°/s 占比</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>高高原次数</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>高高原占比</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>疑似接地前反向蹬舵次数</t>
-        </is>
-      </c>
+    <row r="1" spans="1:13" ht="96" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1.354279523293608E-4</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" s="3">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" s="3">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2" s="3">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" s="4"/>
+      <c r="B3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3">
+        <v>1.354279523293608E-4</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" s="3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3" s="3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" s="4"/>
+      <c r="B4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1.354279523293608E-4</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4" s="3">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5"/>
+      <c r="B5"/>
+      <c r="C5"/>
+      <c r="D5" s="3"/>
+      <c r="E5"/>
+      <c r="F5" s="3"/>
+      <c r="G5"/>
+      <c r="H5" s="3"/>
+      <c r="I5"/>
+      <c r="J5" s="3"/>
+      <c r="K5"/>
+      <c r="L5" s="3"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6"/>
+      <c r="B6"/>
+      <c r="C6"/>
+      <c r="D6" s="3"/>
+      <c r="E6"/>
+      <c r="F6" s="3"/>
+      <c r="G6"/>
+      <c r="H6" s="3"/>
+      <c r="I6"/>
+      <c r="J6" s="3"/>
+      <c r="K6"/>
+      <c r="L6" s="3"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A7"/>
+      <c r="B7"/>
+      <c r="C7"/>
+      <c r="D7" s="3"/>
+      <c r="E7"/>
+      <c r="F7" s="3"/>
+      <c r="G7"/>
+      <c r="H7" s="3"/>
+      <c r="I7"/>
+      <c r="J7" s="3"/>
+      <c r="K7"/>
+      <c r="L7" s="3"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8"/>
+      <c r="B8"/>
+      <c r="C8"/>
+      <c r="D8" s="3"/>
+      <c r="E8"/>
+      <c r="F8" s="3"/>
+      <c r="G8"/>
+      <c r="H8" s="3"/>
+      <c r="I8"/>
+      <c r="J8" s="3"/>
+      <c r="K8"/>
+      <c r="L8" s="3"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9"/>
+      <c r="B9"/>
+      <c r="C9"/>
+      <c r="D9" s="3"/>
+      <c r="E9"/>
+      <c r="F9" s="3"/>
+      <c r="G9"/>
+      <c r="H9" s="3"/>
+      <c r="I9"/>
+      <c r="J9" s="3"/>
+      <c r="K9"/>
+      <c r="L9" s="3"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10"/>
+      <c r="B10"/>
+      <c r="C10"/>
+      <c r="D10" s="3"/>
+      <c r="E10"/>
+      <c r="F10" s="3"/>
+      <c r="G10"/>
+      <c r="H10" s="3"/>
+      <c r="I10"/>
+      <c r="J10" s="3"/>
+      <c r="K10"/>
+      <c r="L10" s="3"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11"/>
+      <c r="B11"/>
+      <c r="C11"/>
+      <c r="D11" s="3"/>
+      <c r="E11"/>
+      <c r="F11" s="3"/>
+      <c r="G11"/>
+      <c r="H11" s="3"/>
+      <c r="I11"/>
+      <c r="J11" s="3"/>
+      <c r="K11"/>
+      <c r="L11" s="3"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A12"/>
+      <c r="B12"/>
+      <c r="C12"/>
+      <c r="D12" s="3"/>
+      <c r="E12"/>
+      <c r="F12" s="3"/>
+      <c r="G12"/>
+      <c r="H12" s="3"/>
+      <c r="I12"/>
+      <c r="J12" s="3"/>
+      <c r="K12"/>
+      <c r="L12" s="3"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13"/>
+      <c r="B13"/>
+      <c r="C13"/>
+      <c r="D13" s="3"/>
+      <c r="E13"/>
+      <c r="F13" s="3"/>
+      <c r="G13"/>
+      <c r="H13" s="3"/>
+      <c r="I13"/>
+      <c r="J13" s="3"/>
+      <c r="K13"/>
+      <c r="L13" s="3"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14"/>
+      <c r="B14"/>
+      <c r="C14"/>
+      <c r="D14" s="3"/>
+      <c r="E14"/>
+      <c r="F14" s="3"/>
+      <c r="G14"/>
+      <c r="H14" s="3"/>
+      <c r="I14"/>
+      <c r="J14" s="3"/>
+      <c r="K14"/>
+      <c r="L14" s="3"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15"/>
+      <c r="B15"/>
+      <c r="C15"/>
+      <c r="D15" s="3"/>
+      <c r="E15"/>
+      <c r="F15" s="3"/>
+      <c r="G15"/>
+      <c r="H15" s="3"/>
+      <c r="I15"/>
+      <c r="J15" s="3"/>
+      <c r="K15"/>
+      <c r="L15" s="3"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16"/>
+      <c r="B16"/>
+      <c r="C16"/>
+      <c r="D16" s="3"/>
+      <c r="E16"/>
+      <c r="F16" s="3"/>
+      <c r="G16"/>
+      <c r="H16" s="3"/>
+      <c r="I16"/>
+      <c r="J16" s="3"/>
+      <c r="K16"/>
+      <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17"/>
+      <c r="B17"/>
+      <c r="C17"/>
+      <c r="D17" s="3"/>
+      <c r="E17"/>
+      <c r="F17" s="3"/>
+      <c r="G17"/>
+      <c r="H17" s="3"/>
+      <c r="I17"/>
+      <c r="J17" s="3"/>
+      <c r="K17"/>
+      <c r="L17" s="3"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:A4"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>